<commit_message>
feat: agregar campo Codigo de Activo Fijo a los equipos
Se agrega como campo opcional en alta/edicion/detalle, busqueda y
exportacion de reportes, carga/actualizacion masiva por Excel, y en
las cartas de entrega/devolucion en PDF.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wwwroot/plantilla_actualizacion_equipos.xlsx
+++ b/wwwroot/plantilla_actualizacion_equipos.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -536,6 +536,7 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -612,6 +613,11 @@
       <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Observaciones</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>CodigoActivoFijo</t>
         </is>
       </c>
     </row>
@@ -628,6 +634,7 @@
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="7" t="n"/>
@@ -642,6 +649,7 @@
       <c r="J6" s="9" t="n"/>
       <c r="K6" s="7" t="n"/>
       <c r="L6" s="7" t="n"/>
+      <c r="M6" s="7" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="n"/>
@@ -656,6 +664,7 @@
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="n"/>
+      <c r="M7" s="4" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="7" t="n"/>
@@ -670,6 +679,7 @@
       <c r="J8" s="9" t="n"/>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="n"/>
@@ -684,6 +694,7 @@
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="4" t="n"/>
+      <c r="M9" s="4" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="7" t="n"/>
@@ -698,6 +709,7 @@
       <c r="J10" s="9" t="n"/>
       <c r="K10" s="7" t="n"/>
       <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="4" t="n"/>
@@ -712,6 +724,7 @@
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="4" t="n"/>
       <c r="L11" s="4" t="n"/>
+      <c r="M11" s="4" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="7" t="n"/>
@@ -726,6 +739,7 @@
       <c r="J12" s="9" t="n"/>
       <c r="K12" s="7" t="n"/>
       <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="4" t="n"/>
@@ -740,6 +754,7 @@
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="4" t="n"/>
       <c r="L13" s="4" t="n"/>
+      <c r="M13" s="4" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="7" t="n"/>
@@ -754,6 +769,7 @@
       <c r="J14" s="9" t="n"/>
       <c r="K14" s="7" t="n"/>
       <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="4" t="n"/>
@@ -768,6 +784,7 @@
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="4" t="n"/>
       <c r="L15" s="4" t="n"/>
+      <c r="M15" s="4" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="7" t="n"/>
@@ -782,6 +799,7 @@
       <c r="J16" s="9" t="n"/>
       <c r="K16" s="7" t="n"/>
       <c r="L16" s="7" t="n"/>
+      <c r="M16" s="7" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="4" t="n"/>
@@ -796,6 +814,7 @@
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="4" t="n"/>
       <c r="L17" s="4" t="n"/>
+      <c r="M17" s="4" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="7" t="n"/>
@@ -810,6 +829,7 @@
       <c r="J18" s="9" t="n"/>
       <c r="K18" s="7" t="n"/>
       <c r="L18" s="7" t="n"/>
+      <c r="M18" s="7" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="4" t="n"/>
@@ -824,6 +844,7 @@
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="4" t="n"/>
       <c r="L19" s="4" t="n"/>
+      <c r="M19" s="4" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="7" t="n"/>
@@ -838,6 +859,7 @@
       <c r="J20" s="9" t="n"/>
       <c r="K20" s="7" t="n"/>
       <c r="L20" s="7" t="n"/>
+      <c r="M20" s="7" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="n"/>
@@ -852,6 +874,7 @@
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="4" t="n"/>
       <c r="L21" s="4" t="n"/>
+      <c r="M21" s="4" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="7" t="n"/>
@@ -866,6 +889,7 @@
       <c r="J22" s="9" t="n"/>
       <c r="K22" s="7" t="n"/>
       <c r="L22" s="7" t="n"/>
+      <c r="M22" s="7" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="n"/>
@@ -880,6 +904,7 @@
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="4" t="n"/>
       <c r="L23" s="4" t="n"/>
+      <c r="M23" s="4" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="7" t="n"/>
@@ -894,11 +919,12 @@
       <c r="J24" s="9" t="n"/>
       <c r="K24" s="7" t="n"/>
       <c r="L24" s="7" t="n"/>
+      <c r="M24" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="K5:K24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Estado inválido" error="Use: Bodega, Asignado, Prestamo, EnGarantia o Baja" type="list">

</xml_diff>